<commit_message>
Solucion de numeros de telefono
</commit_message>
<xml_diff>
--- a/public/Clientes EOR.xlsx
+++ b/public/Clientes EOR.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cristian\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cristian\Documents\S&amp;P\Documentos automatizacion\EOR\Web facturación\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{594E6F1C-1CEA-406F-970F-6E63138EAA11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4CB268-9AEA-4C9C-B4F5-CC120B6D27A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF91D570-95FD-454D-833F-60C60A348C95}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="171">
   <si>
     <t>Nombre tercero</t>
   </si>
@@ -128,9 +128,6 @@
     <t>Atlanta</t>
   </si>
   <si>
-    <t>470-4010092-100</t>
-  </si>
-  <si>
     <t>ELEPHANT</t>
   </si>
   <si>
@@ -164,9 +161,6 @@
     <t>Denver</t>
   </si>
   <si>
-    <t>252-3065772-</t>
-  </si>
-  <si>
     <t>GLOBAL EXPANSION</t>
   </si>
   <si>
@@ -197,9 +191,6 @@
     <t>Downers grove</t>
   </si>
   <si>
-    <t>1-6309716453-</t>
-  </si>
-  <si>
     <t>FLEXCO</t>
   </si>
   <si>
@@ -266,9 +257,6 @@
     <t>ESTADOS UNIDOS</t>
   </si>
   <si>
-    <t>1817-9453584-</t>
-  </si>
-  <si>
     <t>MKD</t>
   </si>
   <si>
@@ -284,9 +272,6 @@
     <t>TALLIN</t>
   </si>
   <si>
-    <t>372-5019568-</t>
-  </si>
-  <si>
     <t>SIFFI</t>
   </si>
   <si>
@@ -302,9 +287,6 @@
     <t>Topeka</t>
   </si>
   <si>
-    <t>913-4221888-</t>
-  </si>
-  <si>
     <t>NAZDAR</t>
   </si>
   <si>
@@ -320,9 +302,6 @@
     <t>Madrid</t>
   </si>
   <si>
-    <t>634-9157518-</t>
-  </si>
-  <si>
     <t>NEO</t>
   </si>
   <si>
@@ -368,9 +347,6 @@
     <t>SAN FRANCISCO</t>
   </si>
   <si>
-    <t>601-7426386-</t>
-  </si>
-  <si>
     <t>REMOFIRST</t>
   </si>
   <si>
@@ -386,9 +362,6 @@
     <t>Hertogenbosch</t>
   </si>
   <si>
-    <t>31-97010286-</t>
-  </si>
-  <si>
     <t>ROOT CAPITAL INC</t>
   </si>
   <si>
@@ -416,9 +389,6 @@
     <t>Chesire</t>
   </si>
   <si>
-    <t>601-27940535-000</t>
-  </si>
-  <si>
     <t>EDRINGTON</t>
   </si>
   <si>
@@ -476,9 +446,6 @@
     <t>Washington Us</t>
   </si>
   <si>
-    <t>1-3609917464-</t>
-  </si>
-  <si>
     <t>Mes vencido</t>
   </si>
   <si>
@@ -552,6 +519,42 @@
   </si>
   <si>
     <t>C1061 - ELEPHANT</t>
+  </si>
+  <si>
+    <t>(31) 97010286</t>
+  </si>
+  <si>
+    <t>(601) 0000000</t>
+  </si>
+  <si>
+    <t>(634) 9157518</t>
+  </si>
+  <si>
+    <t>(913) 4221888</t>
+  </si>
+  <si>
+    <t>(372) 5019568</t>
+  </si>
+  <si>
+    <t>(1817) 9453584</t>
+  </si>
+  <si>
+    <t>(1) 6309716453</t>
+  </si>
+  <si>
+    <t>(470) 4010092 - Ext. 100</t>
+  </si>
+  <si>
+    <t>(252) 3065772</t>
+  </si>
+  <si>
+    <t>(601) 7426386</t>
+  </si>
+  <si>
+    <t>(601) 27940535-000</t>
+  </si>
+  <si>
+    <t>(1) 3609917464</t>
   </si>
 </sst>
 </file>
@@ -655,27 +658,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1066,7 +1049,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>10</v>
@@ -1098,7 +1081,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>19</v>
@@ -1131,7 +1114,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>24</v>
@@ -1146,339 +1129,339 @@
         <v>27</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>29</v>
       </c>
       <c r="K4" s="3"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="4" t="s">
+      <c r="H5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>35</v>
       </c>
       <c r="K5" s="3"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>41</v>
       </c>
       <c r="K6" s="3"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="F7" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>46</v>
-      </c>
       <c r="I7" s="3" t="s">
         <v>17</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="K7" s="3"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="F8" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J8" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>52</v>
       </c>
       <c r="K8" s="3"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="F9" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="J9" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="K9" s="5" t="s">
         <v>56</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="F10" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J10" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>64</v>
       </c>
       <c r="K10" s="3"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="F11" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J11" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>69</v>
       </c>
       <c r="K11" s="3"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="F12" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J12" s="3" t="s">
         <v>71</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>75</v>
       </c>
       <c r="K12" s="3"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J13" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="K13" s="3"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>86</v>
+        <v>162</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>15</v>
@@ -1490,28 +1473,28 @@
         <v>17</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="K14" s="3"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>92</v>
+        <v>161</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>15</v>
@@ -1523,28 +1506,28 @@
         <v>17</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="K15" s="3"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>14</v>
+        <v>160</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>15</v>
@@ -1556,28 +1539,28 @@
         <v>17</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="K16" s="3"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>14</v>
+        <v>160</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>15</v>
@@ -1589,28 +1572,28 @@
         <v>17</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="K17" s="3"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>108</v>
+        <v>168</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>15</v>
@@ -1622,31 +1605,31 @@
         <v>17</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="K18" s="3"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>114</v>
+        <v>159</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>16</v>
@@ -1655,28 +1638,28 @@
         <v>17</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="K19" s="3"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>14</v>
+        <v>160</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>15</v>
@@ -1688,28 +1671,28 @@
         <v>17</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="K20" s="3"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>124</v>
+        <v>169</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>15</v>
@@ -1721,28 +1704,28 @@
         <v>17</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="K21" s="3"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>14</v>
+        <v>160</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>15</v>
@@ -1754,28 +1737,28 @@
         <v>17</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="K22" s="3"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>14</v>
+        <v>160</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>15</v>
@@ -1787,26 +1770,26 @@
         <v>17</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="K23" s="3"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="6"/>
       <c r="B24" s="3" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>14</v>
+        <v>160</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>15</v>
@@ -1818,28 +1801,28 @@
         <v>17</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="K24" s="3"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>144</v>
+        <v>170</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>15</v>
@@ -1848,26 +1831,26 @@
         <v>16</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="K25" s="3"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K25" xr:uid="{63C90589-8B95-422C-99C5-33C3FF9C7ADA}"/>
-  <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="5" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J7:K7">
-    <cfRule type="duplicateValues" dxfId="4" priority="3"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="3" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A25">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J7:K7">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Cambio de nombre del cliente BUBBLE
</commit_message>
<xml_diff>
--- a/public/Clientes EOR.xlsx
+++ b/public/Clientes EOR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cristian\Documents\S&amp;P\Documentos automatizacion\EOR\Web facturación\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4CB268-9AEA-4C9C-B4F5-CC120B6D27A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E4DF989-7DA8-48FB-9AF8-D1A4BBD25136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF91D570-95FD-454D-833F-60C60A348C95}"/>
   </bookViews>
@@ -113,9 +113,6 @@
     <t>Sao Paulo</t>
   </si>
   <si>
-    <t>BUBBLE BPM INC</t>
-  </si>
-  <si>
     <t>ELEPHANT PROPERTY MANAGEMENT LLC</t>
   </si>
   <si>
@@ -555,6 +552,9 @@
   </si>
   <si>
     <t>(1) 3609917464</t>
+  </si>
+  <si>
+    <t>BUBBLE DO BRASIL</t>
   </si>
 </sst>
 </file>
@@ -1049,7 +1049,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>10</v>
@@ -1081,7 +1081,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>19</v>
@@ -1108,528 +1108,528 @@
         <v>17</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>23</v>
+        <v>170</v>
       </c>
       <c r="K3" s="3"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="K4" s="3"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G5" s="4" t="s">
+      <c r="H5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="K5" s="3"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>39</v>
       </c>
       <c r="K6" s="3"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>44</v>
-      </c>
       <c r="I7" s="3" t="s">
         <v>17</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K7" s="3"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J8" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="K8" s="3"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" s="4" t="s">
+      <c r="J9" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="K9" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J10" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>61</v>
       </c>
       <c r="K10" s="3"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J11" s="3" t="s">
         <v>65</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>66</v>
       </c>
       <c r="K11" s="3"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J12" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="K12" s="3"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J13" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>76</v>
       </c>
       <c r="K13" s="3"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="D14" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J14" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="K14" s="3"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="F15" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J15" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="K15" s="3"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>91</v>
       </c>
       <c r="K16" s="3"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="E17" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="F17" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J17" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>96</v>
       </c>
       <c r="K17" s="3"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="F18" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J18" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>101</v>
       </c>
       <c r="K18" s="3"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B19" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>105</v>
-      </c>
       <c r="F19" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>16</v>
@@ -1638,203 +1638,203 @@
         <v>17</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K19" s="3"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="F20" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J20" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>110</v>
       </c>
       <c r="K20" s="3"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="D21" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="F21" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J21" s="3" t="s">
         <v>114</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>115</v>
       </c>
       <c r="K21" s="3"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J22" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I22" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J22" s="3" t="s">
-        <v>119</v>
       </c>
       <c r="K22" s="3"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B23" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="F23" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J23" s="3" t="s">
         <v>123</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J23" s="3" t="s">
-        <v>124</v>
       </c>
       <c r="K23" s="3"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="6"/>
       <c r="B24" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="D24" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="F24" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J24" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="K24" s="3"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="E25" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="F25" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I25" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="F25" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I25" s="4" t="s">
+      <c r="J25" s="3" t="s">
         <v>134</v>
-      </c>
-      <c r="J25" s="3" t="s">
-        <v>135</v>
       </c>
       <c r="K25" s="3"/>
     </row>

</xml_diff>